<commit_message>
Añadir el campo de intolerancias a los jugadores
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/plantilla-modelo.xlsx
+++ b/public/plantillas/plantilla-modelo.xlsx
@@ -397,14 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,6 +415,9 @@
       <c r="E1" t="str">
         <v>DNI</v>
       </c>
+      <c r="F1" t="str">
+        <v>Intolerancias</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -439,10 +435,13 @@
       <c r="E2" t="str">
         <v>00000000A</v>
       </c>
+      <c r="F2" t="str">
+        <v>Lactosa</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>